<commit_message>
feat(productos): Kit de Tareas Catering v2.0 (346 tareas) y Chocolatería v2.0 (338, criterio de templado en las 3 coberturas) — motor 2.4 + contenido propio; molde P4 normalizado (DV, contador sin rótulos); idempotencia 0, censo 0, gate offline 11/11
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-catering/01-apertura-cierre.xlsx
+++ b/astro-site/public/dl/kit-tareas-catering/01-apertura-cierre.xlsx
@@ -88,7 +88,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -131,8 +131,13 @@
         <bgColor rgb="00EFEBE9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -154,11 +159,55 @@
         <color rgb="00E0E0E0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0E0E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0E0E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -200,6 +249,17 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -576,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -651,9 +711,45 @@
     </row>
     <row r="13"/>
     <row r="14">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-tareas-catering · info@aichef.pro</t>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Seguridad y vida útil:</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>▸ La primera sección de «Producción» es de higiene personal y de arranque seguro de la cocina: campana primero, comprobación del gas después y sólo entonces hornos, sous-vide y freidora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>▸ El pescado que se sirve crudo o semicrudo (ceviche, tartar, marinados, ahumado en frío) necesita congelación previa: ≥24 h a −20 °C o 15 h a −35 °C. Pide el certificado al proveedor y anota el lote.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>▸ Al pie de la hoja tienes una tabla editable de vida útil en congelación por familia: ajústala a tu producto y a tu proveedor. Está fuera del contador porque es una referencia, no una tarea.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Diseñado por John Guerrero — chef y consultor gastronómico desde 2010, en cocina desde los 17 años · johnguerrero.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Versión 2.0 · agosto 2026 · aichef.pro/kit-tareas-catering · info@aichef.pro</t>
         </is>
       </c>
     </row>
@@ -678,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -905,7 +1001,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Producción D-1 (día anterior)</t>
+          <t>Higiene personal y arranque seguro de la cocina</t>
         </is>
       </c>
     </row>
@@ -952,7 +1048,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Recepción y control de mercancía: temperaturas, cantidades, calidad</t>
+          <t>Uniforme y calzado de trabajo limpios, delantal cambiado y pelo recogido (gorro o redecilla)</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
@@ -971,7 +1067,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Almacenar correctamente: refrigeración, congelación, secos</t>
+          <t>Sin anillos, reloj ni pulseras; uñas cortas, limpias y sin esmalte</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
@@ -990,7 +1086,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Mise en place de salsas base, fondos y reducciones</t>
+          <t>Heridas y cortes cubiertos con apósito impermeable de color visible y guante encima</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
@@ -1009,7 +1105,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Preparar marinados, adobos y maceraciones que requieran tiempo</t>
+          <t>Lavado de manos al entrar y en cada cambio de tarea: jabón, agua caliente y papel de un solo uso</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
@@ -1028,7 +1124,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Elaborar masas, bases de tartas y postres que necesiten reposo</t>
+          <t>Declarar síntomas digestivos o respiratorios: quien los tenga no manipula alimentos</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
@@ -1047,7 +1143,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Preparar pre-cocciones: confitados, braseados, sous-vide</t>
+          <t>Encender la campana extractora y ventilar la cocina ANTES de encender nada más</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
@@ -1066,7 +1162,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Cortar y porcionar proteínas según ficha técnica</t>
+          <t>Si la cocina tiene gas: abrir la llave general y comprobar que NO huele a gas; si huele, no enciendas nada, ventila y avisa al mantenedor</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -1085,7 +1181,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Preparar guarniciones y vegetales: lavar, cortar, blanquear</t>
+          <t>Encender hornos, sous-vide, abatidor y freidora sólo después de la campana y del control del gas</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -1099,95 +1195,113 @@
       <c r="G24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Etiquetar todo con producto, fecha, lote y alérgenos</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>Producción</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="n"/>
-      <c r="E25" s="12" t="n"/>
-      <c r="F25" s="11" t="n"/>
-      <c r="G25" s="13" t="n"/>
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Producción D-1 (día anterior)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>Organizar cámaras por orden de carga para transporte</t>
-        </is>
-      </c>
-      <c r="C26" s="14" t="inlineStr">
-        <is>
-          <t>Producción</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="n"/>
-      <c r="E26" s="12" t="n"/>
-      <c r="F26" s="11" t="n"/>
-      <c r="G26" s="13" t="n"/>
-    </row>
-    <row r="27"/>
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Recepción y control de mercancía: temperaturas, cantidades, calidad</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="13" t="n"/>
+    </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>Producción día D (día del evento)</t>
-        </is>
-      </c>
+      <c r="A28" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Almacenar correctamente (refrigeración 0-4 °C, congelación ≤ −18 °C, secos) y etiquetar con la fecha: la vida útil por familia está en la tabla del pie de esta hoja</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Tarea</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Zona</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Responsable</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Hora</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>Notas</t>
-        </is>
-      </c>
+      <c r="A29" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Mise en place de salsas base, fondos y reducciones</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="13" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Verificar temperaturas de cámaras y producto almacenado</t>
+          <t>Preparar marinados, adobos y maceraciones que requieran tiempo</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
@@ -1202,11 +1316,11 @@
     </row>
     <row r="31">
       <c r="A31" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Completar elaboraciones finales: hornear, grillar, freír</t>
+          <t>Elaborar masas, bases de tartas y postres que necesiten reposo</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
@@ -1221,11 +1335,11 @@
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Preparar salsas y aderezos de última hora</t>
+          <t>Preparar pre-cocciones: confitados, braseados, sous-vide</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -1240,11 +1354,11 @@
     </row>
     <row r="33">
       <c r="A33" s="8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Emplatado previo de entrantes fríos y canapés</t>
+          <t>Cortar y porcionar proteínas según ficha técnica</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -1259,11 +1373,11 @@
     </row>
     <row r="34">
       <c r="A34" s="8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Montar bandejas de presentación y centros de mesa comestibles</t>
+          <t>Pescado que se servirá crudo o semicrudo (ceviche, tartar, marinados, ahumado en frío) — prevención de ANISAKIS: exigir al proveedor el certificado de congelación previa (≥24 h a −20 °C, o 15 h a −35 °C) o congelarlo tú, y anotar el lote</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -1278,11 +1392,11 @@
     </row>
     <row r="35">
       <c r="A35" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>Verificar cantidades vs. ficha del evento (check cruzado)</t>
+          <t>Preparar guarniciones y vegetales: lavar, cortar y blanquear. Los que se sirvan CRUDOS, desinfectar con lejía apta para uso alimentario según la dosis del fabricante (habitual: 70 ppm, 5 min) y ACLARAR con agua potable abundante</t>
         </is>
       </c>
       <c r="C35" s="14" t="inlineStr">
@@ -1297,11 +1411,11 @@
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Empaquetado en GN y contenedores isotérmicos etiquetados</t>
+          <t>Etiquetar todo con producto, fecha, lote y alérgenos</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
@@ -1316,11 +1430,11 @@
     </row>
     <row r="37">
       <c r="A37" s="8" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>Control de temperatura pre-transporte (registrar en APPCC)</t>
+          <t>Organizar cámaras por orden de carga para transporte</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
@@ -1333,96 +1447,566 @@
       <c r="F37" s="11" t="n"/>
       <c r="G37" s="13" t="n"/>
     </row>
-    <row r="38">
-      <c r="A38" s="8" t="n">
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Producción día D (día del evento)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Comprobar que las cámaras han funcionado toda la noche y registrar la temperatura (refrigeración 0-4 °C / congelación ≤ −18 °C) — anota la lectura: ____ °C. Si hay desviación, no cargues el género hasta valorarlo</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="13" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Completar elaboraciones finales: hornear, grillar, freír</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="13" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Preparar salsas y aderezos de última hora</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="12" t="n"/>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="13" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Emplatado previo de entrantes fríos y canapés</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="n"/>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="11" t="n"/>
+      <c r="G44" s="13" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Montar bandejas de presentación y centros de mesa comestibles</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="11" t="n"/>
+      <c r="G45" s="13" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Verificar cantidades vs. ficha del evento (check cruzado)</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="12" t="n"/>
+      <c r="F46" s="11" t="n"/>
+      <c r="G46" s="13" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Empaquetado en GN y contenedores isotérmicos etiquetados</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="n"/>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="11" t="n"/>
+      <c r="G47" s="13" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Control de temperatura antes de cargar — anota la lectura: ____ °C (si tienes el Pack APPCC, regístrala en su hoja de temperaturas; si no, en la columna «Notas»)</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="12" t="n"/>
+      <c r="F48" s="11" t="n"/>
+      <c r="G48" s="13" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B49" s="9" t="inlineStr">
         <is>
           <t>Verificar utensilios, menaje y material de servicio empaquetado</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr">
-        <is>
-          <t>Producción</t>
-        </is>
-      </c>
-      <c r="D38" s="11" t="n"/>
-      <c r="E38" s="12" t="n"/>
-      <c r="F38" s="11" t="n"/>
-      <c r="G38" s="13" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="n">
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="n"/>
+      <c r="E49" s="12" t="n"/>
+      <c r="F49" s="11" t="n"/>
+      <c r="G49" s="13" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>Anotar las mermas de producción del día (producto, cantidad y motivo): es el dato que corrige el escandallo del próximo evento</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="12" t="n"/>
+      <c r="F50" s="11" t="n"/>
+      <c r="G50" s="13" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
         <is>
           <t>Limpieza y desinfección de la zona de producción post-carga</t>
         </is>
       </c>
-      <c r="C39" s="16" t="inlineStr">
+      <c r="C51" s="16" t="inlineStr">
         <is>
           <t>Limpieza</t>
         </is>
       </c>
-      <c r="D39" s="11" t="n"/>
-      <c r="E39" s="12" t="n"/>
-      <c r="F39" s="11" t="n"/>
-      <c r="G39" s="13" t="n"/>
-    </row>
-    <row r="40">
-      <c r="B40" s="18" t="inlineStr">
+      <c r="D51" s="11" t="n"/>
+      <c r="E51" s="12" t="n"/>
+      <c r="F51" s="11" t="n"/>
+      <c r="G51" s="13" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="18" t="inlineStr">
         <is>
           <t>Tareas completadas:</t>
         </is>
       </c>
-      <c r="C40">
-        <f>COUNTIF(E6:E39,"✓")</f>
-        <v>2.0</v>
-      </c>
-      <c r="D40" t="inlineStr">
+      <c r="C52">
+        <f>COUNTIFS(B6:B51,"?*",E6:E51,"✓")-COUNTIFS(B6:B51,"Tarea",E6:E51,"✓")</f>
+        <v>0.0</v>
+      </c>
+      <c r="D52" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="E40">
-        <f>COUNTIF(B6:B39,"?*")</f>
-        <v>30.0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+      <c r="E52">
+        <f>COUNTIF(B6:B51,"?*")-COUNTIF(B6:B51,"Tarea")-COUNTIF(E6:E51,"N/A")</f>
+        <v>38.0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>Firma responsable: _________________  Fecha: ___/___/______</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="17" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>VIDA ÚTIL ORIENTATIVA EN CONGELACIÓN A −18 °C — ajústala a tu producto y a tu proveedor</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="n"/>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Familia</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Vida útil</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="E56" s="19" t="n"/>
+      <c r="F56" s="19" t="n"/>
+      <c r="G56" s="20" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n"/>
+      <c r="B57" s="21" t="inlineStr">
+        <is>
+          <t>Carnes rojas y aves crudas, en pieza</t>
+        </is>
+      </c>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>6-12 meses</t>
+        </is>
+      </c>
+      <c r="D57" s="23" t="inlineStr">
+        <is>
+          <t>Porciona ANTES de congelar: descongelar y volver a congelar no se hace</t>
+        </is>
+      </c>
+      <c r="E57" s="19" t="n"/>
+      <c r="F57" s="19" t="n"/>
+      <c r="G57" s="20" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n"/>
+      <c r="B58" s="21" t="inlineStr">
+        <is>
+          <t>Carne picada y preparados de carne</t>
+        </is>
+      </c>
+      <c r="C58" s="22" t="inlineStr">
+        <is>
+          <t>3 meses</t>
+        </is>
+      </c>
+      <c r="D58" s="23" t="inlineStr">
+        <is>
+          <t>Más superficie expuesta: se enrancia y se oxida mucho antes que la pieza entera</t>
+        </is>
+      </c>
+      <c r="E58" s="19" t="n"/>
+      <c r="F58" s="19" t="n"/>
+      <c r="G58" s="20" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n"/>
+      <c r="B59" s="21" t="inlineStr">
+        <is>
+          <t>Pescado blanco y marisco crudo</t>
+        </is>
+      </c>
+      <c r="C59" s="22" t="inlineStr">
+        <is>
+          <t>3-6 meses</t>
+        </is>
+      </c>
+      <c r="D59" s="23" t="inlineStr">
+        <is>
+          <t>El tratamiento antianisakis (≥24 h a −20 °C) no sustituye a esta vida útil: se cuentan por separado</t>
+        </is>
+      </c>
+      <c r="E59" s="19" t="n"/>
+      <c r="F59" s="19" t="n"/>
+      <c r="G59" s="20" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n"/>
+      <c r="B60" s="21" t="inlineStr">
+        <is>
+          <t>Pescado azul (salmón, atún, boquerón)</t>
+        </is>
+      </c>
+      <c r="C60" s="22" t="inlineStr">
+        <is>
+          <t>2-3 meses</t>
+        </is>
+      </c>
+      <c r="D60" s="23" t="inlineStr">
+        <is>
+          <t>La grasa se enrancia aunque esté congelado: es el que antes se estropea</t>
+        </is>
+      </c>
+      <c r="E60" s="19" t="n"/>
+      <c r="F60" s="19" t="n"/>
+      <c r="G60" s="20" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="n"/>
+      <c r="B61" s="21" t="inlineStr">
+        <is>
+          <t>Fondos, salsas, cremas y reducciones propias</t>
+        </is>
+      </c>
+      <c r="C61" s="22" t="inlineStr">
+        <is>
+          <t>3 meses</t>
+        </is>
+      </c>
+      <c r="D61" s="23" t="inlineStr">
+        <is>
+          <t>Etiqueta con la fecha de producción Y la de congelación: la vida útil se cuenta desde la de congelación</t>
+        </is>
+      </c>
+      <c r="E61" s="19" t="n"/>
+      <c r="F61" s="19" t="n"/>
+      <c r="G61" s="20" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="n"/>
+      <c r="B62" s="21" t="inlineStr">
+        <is>
+          <t>Masas crudas, bases de tarta y hojaldre</t>
+        </is>
+      </c>
+      <c r="C62" s="22" t="inlineStr">
+        <is>
+          <t>1-2 meses</t>
+        </is>
+      </c>
+      <c r="D62" s="23" t="inlineStr">
+        <is>
+          <t>La levadura pierde fuerza: después sube mal aunque siga siendo seguro</t>
+        </is>
+      </c>
+      <c r="E62" s="19" t="n"/>
+      <c r="F62" s="19" t="n"/>
+      <c r="G62" s="20" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="n"/>
+      <c r="B63" s="21" t="inlineStr">
+        <is>
+          <t>Pan y bollería ya horneados</t>
+        </is>
+      </c>
+      <c r="C63" s="22" t="inlineStr">
+        <is>
+          <t>1-3 meses</t>
+        </is>
+      </c>
+      <c r="D63" s="23" t="inlineStr">
+        <is>
+          <t>Pierde textura antes que seguridad; regenera en horno, nunca en microondas</t>
+        </is>
+      </c>
+      <c r="E63" s="19" t="n"/>
+      <c r="F63" s="19" t="n"/>
+      <c r="G63" s="20" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n"/>
+      <c r="B64" s="21" t="inlineStr">
+        <is>
+          <t>Canapés y bocados montados</t>
+        </is>
+      </c>
+      <c r="C64" s="22" t="inlineStr">
+        <is>
+          <t>1 mes</t>
+        </is>
+      </c>
+      <c r="D64" s="23" t="inlineStr">
+        <is>
+          <t>Sólo los que admiten congelación: con mayonesa, gelatina o nata montada NO se congelan</t>
+        </is>
+      </c>
+      <c r="E64" s="19" t="n"/>
+      <c r="F64" s="19" t="n"/>
+      <c r="G64" s="20" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="n"/>
+      <c r="B65" s="21" t="inlineStr">
+        <is>
+          <t>Verdura blanqueada, purés y guarniciones</t>
+        </is>
+      </c>
+      <c r="C65" s="22" t="inlineStr">
+        <is>
+          <t>8-12 meses</t>
+        </is>
+      </c>
+      <c r="D65" s="23" t="inlineStr">
+        <is>
+          <t>Blanquea antes de congelar: sin blanquear pierde color y textura en pocas semanas</t>
+        </is>
+      </c>
+      <c r="E65" s="19" t="n"/>
+      <c r="F65" s="19" t="n"/>
+      <c r="G65" s="20" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n"/>
+      <c r="B66" s="21" t="inlineStr">
+        <is>
+          <t>Producto que ya ha salido a un servicio</t>
+        </is>
+      </c>
+      <c r="C66" s="22" t="inlineStr">
+        <is>
+          <t>No congelar</t>
+        </is>
+      </c>
+      <c r="D66" s="23" t="inlineStr">
+        <is>
+          <t>Lo que ha estado expuesto en sala o ha roto la cadena de frío no vuelve al congelador: se retira</t>
+        </is>
+      </c>
+      <c r="E66" s="19" t="n"/>
+      <c r="F66" s="19" t="n"/>
+      <c r="G66" s="20" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
         <is>
           <t>© 2026 AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="20">
+    <mergeCell ref="D63:G63"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="D65:G65"/>
+    <mergeCell ref="D64:G64"/>
+    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="D62:G62"/>
+    <mergeCell ref="D66:G66"/>
+    <mergeCell ref="D61:G61"/>
+    <mergeCell ref="A67:G67"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="D56:G56"/>
     <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="D58:G58"/>
+    <mergeCell ref="D59:G59"/>
+    <mergeCell ref="D60:G60"/>
+    <mergeCell ref="D57:G57"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A53:G53"/>
   </mergeCells>
-  <conditionalFormatting sqref="A6:G39">
+  <conditionalFormatting sqref="A6:G51">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E6="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E6 E7 E8 E9 E10 E11 E12 E13 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Usa ✓, ✗ o —" prompt="Marca ✓ si completada" type="list">
-      <formula1>"✓,✗,—"</formula1>
+    <dataValidation sqref="E6 E7 E8 E9 E10 E11 E12 E13 E17 E18 E19 E20 E21 E22 E23 E24 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." prompt="Marca ✓ si completada" type="list" errorStyle="stop">
+      <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>

</xml_diff>